<commit_message>
Add CO2 T&S 4-45 $/t bar to Full-CCS tornado
Eighth bar on the two Full-CCS panels: sequestered CO2 (623CO2+622X) priced at
4-45 $/tCO2, base 0; span ~0.28 $/L, scale-invariant. Report method table, §2,
and log updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016MjFwwDgUpjrZDZMd1ma7x
</commit_message>
<xml_diff>
--- a/Figure/tornado_sensitivity.xlsx
+++ b/Figure/tornado_sensitivity.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1259,25 +1259,25 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Capacity 85% / 91%</t>
+          <t>CO₂ T&amp;S 4–45 $/t</t>
         </is>
       </c>
       <c r="D31" t="n">
         <v>2.206999917290672</v>
       </c>
       <c r="E31" t="n">
-        <v>2.47530760834593</v>
+        <v>2.234034453758579</v>
       </c>
       <c r="F31" t="n">
-        <v>2.219847435166805</v>
+        <v>2.511138452554633</v>
       </c>
       <c r="G31" t="n">
-        <v>0.2554601731791242</v>
+        <v>0.2771039987960533</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1286,20 +1286,20 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Gray H₂ 1–4 $/kg</t>
+          <t>Capacity 85% / 91%</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1.130706493835227</v>
+        <v>2.206999917290672</v>
       </c>
       <c r="E32" t="n">
-        <v>0.9210666174655715</v>
+        <v>2.47530760834593</v>
       </c>
       <c r="F32" t="n">
-        <v>2.179549555559209</v>
+        <v>2.219847435166805</v>
       </c>
       <c r="G32" t="n">
-        <v>1.258482938093638</v>
+        <v>0.2554601731791242</v>
       </c>
     </row>
     <row r="33">
@@ -1313,20 +1313,20 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Biomass ±50%</t>
+          <t>Gray H₂ 1–4 $/kg</t>
         </is>
       </c>
       <c r="D33" t="n">
         <v>1.130706493835227</v>
       </c>
       <c r="E33" t="n">
-        <v>0.8186793339407283</v>
+        <v>0.9210666174655715</v>
       </c>
       <c r="F33" t="n">
-        <v>1.442733653729725</v>
+        <v>2.179549555559209</v>
       </c>
       <c r="G33" t="n">
-        <v>0.6240543197889967</v>
+        <v>1.258482938093638</v>
       </c>
     </row>
     <row r="34">
@@ -1340,20 +1340,20 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Co-product ±20%</t>
+          <t>Biomass ±50%</t>
         </is>
       </c>
       <c r="D34" t="n">
         <v>1.130706493835227</v>
       </c>
       <c r="E34" t="n">
-        <v>1.377571870021486</v>
+        <v>0.8186793339407283</v>
       </c>
       <c r="F34" t="n">
-        <v>0.8838411176489671</v>
+        <v>1.442733653729725</v>
       </c>
       <c r="G34" t="n">
-        <v>0.4937307523725192</v>
+        <v>0.6240543197889967</v>
       </c>
     </row>
     <row r="35">
@@ -1367,20 +1367,20 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CAPEX ±30%</t>
+          <t>Co-product ±20%</t>
         </is>
       </c>
       <c r="D35" t="n">
         <v>1.130706493835227</v>
       </c>
       <c r="E35" t="n">
-        <v>0.9102710747935859</v>
+        <v>1.377571870021486</v>
       </c>
       <c r="F35" t="n">
-        <v>1.351141912876868</v>
+        <v>0.8838411176489671</v>
       </c>
       <c r="G35" t="n">
-        <v>0.4408708380832816</v>
+        <v>0.4937307523725192</v>
       </c>
     </row>
     <row r="36">
@@ -1394,20 +1394,20 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Electricity ±30%</t>
+          <t>CAPEX ±30%</t>
         </is>
       </c>
       <c r="D36" t="n">
         <v>1.130706493835227</v>
       </c>
       <c r="E36" t="n">
-        <v>1.272592747951792</v>
+        <v>0.9102710747935859</v>
       </c>
       <c r="F36" t="n">
-        <v>0.9888202397186625</v>
+        <v>1.351141912876868</v>
       </c>
       <c r="G36" t="n">
-        <v>0.2837725082331291</v>
+        <v>0.4408708380832816</v>
       </c>
     </row>
     <row r="37">
@@ -1421,19 +1421,73 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Capacity 85% / 91%</t>
+          <t>Electricity ±30%</t>
         </is>
       </c>
       <c r="D37" t="n">
         <v>1.130706493835227</v>
       </c>
       <c r="E37" t="n">
+        <v>1.272592747951792</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.9888202397186625</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.2837725082331291</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>30</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Full-CCS</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CO₂ T&amp;S 4–45 $/t</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1.130706493835227</v>
+      </c>
+      <c r="E38" t="n">
+        <v>1.157741029796421</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1.43484502339866</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.2771039936022397</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>30</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Full-CCS</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Capacity 85% / 91%</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1.130706493835227</v>
+      </c>
+      <c r="E39" t="n">
         <v>1.318935409052217</v>
       </c>
-      <c r="F37" t="n">
+      <c r="F39" t="n">
         <v>1.13971955769316</v>
       </c>
-      <c r="G37" t="n">
+      <c r="G39" t="n">
         <v>0.1792158513590565</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adopt $10/tCO2 CO2 T&S basis for the CCS unit
Tornado: CCS base now carries $10/t T&S via co2_ts_usd_per_ton; T&S bar sweeps
4-45 $/t around it. Full-CCS base MJSP 2.21->2.28 (x1), 1.13->1.20 (x30).
_Scale_Up_Subunits.md CCS MJSP and $/tCO2 recomputed at $10/t (matched-CCS
abatement shape inverts: EGR CO2 pays T&S at any capture rate).
_Scale_Up_Sensitivity.md left T&S-free with a note (stays a 4-45 range).
_Base_Revision.md §4.11 cites Smith IJGGC 2021 for the T&S price range.
funs.py default co2_ts_usd_per_ton=0 unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016MjFwwDgUpjrZDZMd1ma7x
</commit_message>
<xml_diff>
--- a/Figure/tornado_sensitivity.xlsx
+++ b/Figure/tornado_sensitivity.xlsx
@@ -1128,13 +1128,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>2.206999917290672</v>
+        <v>2.274586258460441</v>
       </c>
       <c r="E26" t="n">
-        <v>1.997359869614372</v>
+        <v>2.064946210784141</v>
       </c>
       <c r="F26" t="n">
-        <v>3.255843835713536</v>
+        <v>3.323430176883305</v>
       </c>
       <c r="G26" t="n">
         <v>1.258483966099164</v>
@@ -1155,13 +1155,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2.206999917290672</v>
+        <v>2.274586258460441</v>
       </c>
       <c r="E27" t="n">
-        <v>1.820299884225325</v>
+        <v>1.887886225395094</v>
       </c>
       <c r="F27" t="n">
-        <v>2.593699950356019</v>
+        <v>2.661286291525788</v>
       </c>
       <c r="G27" t="n">
         <v>0.7734000661306941</v>
@@ -1182,13 +1182,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2.206999917290672</v>
+        <v>2.274586258460441</v>
       </c>
       <c r="E28" t="n">
-        <v>1.882923977198296</v>
+        <v>1.950510318368065</v>
       </c>
       <c r="F28" t="n">
-        <v>2.531075857383047</v>
+        <v>2.598662198552816</v>
       </c>
       <c r="G28" t="n">
         <v>0.6481518801847512</v>
@@ -1209,16 +1209,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2.206999917290672</v>
+        <v>2.274586258460441</v>
       </c>
       <c r="E29" t="n">
-        <v>2.45386529513638</v>
+        <v>2.521451636306149</v>
       </c>
       <c r="F29" t="n">
-        <v>1.960134539444964</v>
+        <v>2.027720880614733</v>
       </c>
       <c r="G29" t="n">
-        <v>0.4937307556914161</v>
+        <v>0.4937307556914159</v>
       </c>
     </row>
     <row r="30">
@@ -1236,16 +1236,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2.206999917290672</v>
+        <v>2.274586258460441</v>
       </c>
       <c r="E30" t="n">
-        <v>2.348886174481059</v>
+        <v>2.416472515650828</v>
       </c>
       <c r="F30" t="n">
-        <v>2.065113660100285</v>
+        <v>2.132700001270055</v>
       </c>
       <c r="G30" t="n">
-        <v>0.2837725143807739</v>
+        <v>0.283772514380773</v>
       </c>
     </row>
     <row r="31">
@@ -1263,7 +1263,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2.206999917290672</v>
+        <v>2.274586258460441</v>
       </c>
       <c r="E31" t="n">
         <v>2.234034453758579</v>
@@ -1290,16 +1290,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2.206999917290672</v>
+        <v>2.274586258460441</v>
       </c>
       <c r="E32" t="n">
-        <v>2.47530760834593</v>
+        <v>2.542893949515699</v>
       </c>
       <c r="F32" t="n">
-        <v>2.219847435166805</v>
+        <v>2.287433776336574</v>
       </c>
       <c r="G32" t="n">
-        <v>0.2554601731791242</v>
+        <v>0.2554601731791251</v>
       </c>
     </row>
     <row r="33">
@@ -1317,16 +1317,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1.130706493835227</v>
+        <v>1.198292833738212</v>
       </c>
       <c r="E33" t="n">
-        <v>0.9210666174655715</v>
+        <v>0.9886529573685572</v>
       </c>
       <c r="F33" t="n">
-        <v>2.179549555559209</v>
+        <v>2.247135895462194</v>
       </c>
       <c r="G33" t="n">
-        <v>1.258482938093638</v>
+        <v>1.258482938093637</v>
       </c>
     </row>
     <row r="34">
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1.130706493835227</v>
+        <v>1.198292833738212</v>
       </c>
       <c r="E34" t="n">
-        <v>0.8186793339407283</v>
+        <v>0.886265673843714</v>
       </c>
       <c r="F34" t="n">
-        <v>1.442733653729725</v>
+        <v>1.510319993632711</v>
       </c>
       <c r="G34" t="n">
         <v>0.6240543197889967</v>
@@ -1371,16 +1371,16 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1.130706493835227</v>
+        <v>1.198292833738212</v>
       </c>
       <c r="E35" t="n">
-        <v>1.377571870021486</v>
+        <v>1.445158209924472</v>
       </c>
       <c r="F35" t="n">
-        <v>0.8838411176489671</v>
+        <v>0.9514274575519527</v>
       </c>
       <c r="G35" t="n">
-        <v>0.4937307523725192</v>
+        <v>0.4937307523725193</v>
       </c>
     </row>
     <row r="36">
@@ -1398,13 +1398,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1.130706493835227</v>
+        <v>1.198292833738212</v>
       </c>
       <c r="E36" t="n">
-        <v>0.9102710747935859</v>
+        <v>0.9778574146965716</v>
       </c>
       <c r="F36" t="n">
-        <v>1.351141912876868</v>
+        <v>1.418728252779853</v>
       </c>
       <c r="G36" t="n">
         <v>0.4408708380832816</v>
@@ -1425,16 +1425,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1.130706493835227</v>
+        <v>1.198292833738212</v>
       </c>
       <c r="E37" t="n">
-        <v>1.272592747951792</v>
+        <v>1.340179087854777</v>
       </c>
       <c r="F37" t="n">
-        <v>0.9888202397186625</v>
+        <v>1.056406579621648</v>
       </c>
       <c r="G37" t="n">
-        <v>0.2837725082331291</v>
+        <v>0.2837725082331284</v>
       </c>
     </row>
     <row r="38">
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1.130706493835227</v>
+        <v>1.198292833738212</v>
       </c>
       <c r="E38" t="n">
         <v>1.157741029796421</v>
@@ -1461,7 +1461,7 @@
         <v>1.43484502339866</v>
       </c>
       <c r="G38" t="n">
-        <v>0.2771039936022397</v>
+        <v>0.2771039936022393</v>
       </c>
     </row>
     <row r="39">
@@ -1479,16 +1479,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1.130706493835227</v>
+        <v>1.198292833738212</v>
       </c>
       <c r="E39" t="n">
-        <v>1.318935409052217</v>
+        <v>1.386521748955202</v>
       </c>
       <c r="F39" t="n">
-        <v>1.13971955769316</v>
+        <v>1.207305897596145</v>
       </c>
       <c r="G39" t="n">
-        <v>0.1792158513590565</v>
+        <v>0.1792158513590572</v>
       </c>
     </row>
   </sheetData>

</xml_diff>